<commit_message>
Record May expensas for BONORINO.
Capture the Consorcio Bonorino 82 Mercado Pago transfer so the property workbook tracks its own building fees separately from CIUDAD.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -65,7 +65,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -87,11 +87,55 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -105,6 +149,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -588,14 +635,28 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="H5" s="5" t="n">
+        <v>200340</v>
+      </c>
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
@@ -908,8 +969,8 @@
           <t>TOTAL MES</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="13" t="n"/>
       <c r="D20" s="7">
         <f>SUM(D5:D19)</f>
         <v/>
@@ -1052,16 +1113,44 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
+      <c r="A4" s="9" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Expensas — Cons De Prop E Bonorino 82</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>200340</v>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Transferencia Mercado Pago</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr"/>
+      <c r="H4" s="10" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Op 159022197576 · CUIL 30536004005 · Banco Comafi · Original 200339.05 · ceil</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>

</xml_diff>

<commit_message>
Catalog Mercado Pago expenses for CIUDAD and expand grocery detail.
Classify the extract into fixed rules, load confirmed ALMACEN SOL items by month, and keep pending merchants for confirmation.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -657,8 +657,12 @@
       <c r="H5" s="5" t="n">
         <v>200340</v>
       </c>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
+      <c r="I5" s="5" t="n">
+        <v>219145</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>209393</v>
+      </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
@@ -1153,28 +1157,84 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="4" t="n"/>
+      <c r="A5" s="9" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Expensas — Cons De Prop E Bonorino 82</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>219145</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Transferencia Mercado Pago</t>
+        </is>
+      </c>
       <c r="G5" s="10" t="n"/>
       <c r="H5" s="10" t="n"/>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Desde extracto MP CIUDAD (ceil)</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="4" t="n"/>
+      <c r="A6" s="9" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Expensas — Cons De Prop E Bonorino 82</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>209393</v>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Transferencia Mercado Pago</t>
+        </is>
+      </c>
       <c r="G6" s="10" t="n"/>
       <c r="H6" s="10" t="n"/>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="4" t="n"/>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Desde extracto MP CIUDAD (ceil)</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>

</xml_diff>

<commit_message>
Load expensas from Gmail and map BBVA Visa utility auto-debits.
Confirm Copropi as OHIGGINS, fix CIUDAD expensas periods, and document Edenor/Metrogas/Telecentro débitos on Visa Signature.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -135,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,6 +153,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -548,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gastos 2026 — propiedad independiente</t>
+          <t>Gastos 2026 — propiedad independiente · Edesur = LUZ BONORINO</t>
         </is>
       </c>
     </row>
@@ -674,15 +676,33 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>LUZ</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Edesur</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
+      <c r="G6" s="5" t="n">
+        <v>1685</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>1441</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>2198</v>
+      </c>
       <c r="J6" s="5" t="n"/>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="5" t="n"/>
@@ -1237,37 +1257,109 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="10" t="n"/>
+      <c r="A7" s="14" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>LUZ</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Edesur</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>1685</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Factura digital Gmail / MP</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>3932799</t>
+        </is>
+      </c>
       <c r="H7" s="10" t="n"/>
       <c r="I7" s="4" t="n"/>
       <c r="J7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="A8" s="14" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>LUZ</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Edesur</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>1441</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Factura digital Gmail / MP</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>3932799</t>
+        </is>
+      </c>
       <c r="H8" s="10" t="n"/>
       <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="A9" s="14" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>LUZ</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Edesur</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>2198</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Factura digital Gmail / MP</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>3932799</t>
+        </is>
+      </c>
       <c r="H9" s="10" t="n"/>
       <c r="I9" s="4" t="n"/>
       <c r="J9" s="4" t="n"/>

</xml_diff>

<commit_message>
Cargar expensas BONORINO agosto 2026 ($222.825)
- Matriz 2026 columna Agosto: 222825 (ceil de 222824.05)
- Detalle: Cons De Prop E Bonorino 82 · fecha tentativa 10/08 pendiente extracto MP

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -665,7 +665,9 @@
       <c r="J5" s="5" t="n">
         <v>209393</v>
       </c>
-      <c r="K5" s="5" t="n"/>
+      <c r="K5" s="5" t="n">
+        <v>222825</v>
+      </c>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
@@ -1403,16 +1405,44 @@
       <c r="J10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="A11" s="9" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Expensas — Cons De Prop E Bonorino 82</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>222825</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Transferencia Mercado Pago</t>
+        </is>
+      </c>
       <c r="G11" s="10" t="n"/>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="4" t="n"/>
-      <c r="J11" s="4" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Original 222824.05 · ceil · REVISAR fecha pago (pendiente extracto MP)</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>

</xml_diff>

<commit_message>
Confirmar pago MP expensas BONORINO agosto 2026 (01/09)
- Fecha real 01/09/2026 · Op 175716187231 · $222.825
- Espejo CIUDAD Expensas Consorcios
- Catálogo MP y movimientos cuenta actualizados

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -1406,7 +1406,7 @@
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
-        <v>46244</v>
+        <v>46266</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
@@ -1435,7 +1435,7 @@
       <c r="H11" s="10" t="n"/>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Original 222824.05 · ceil · REVISAR fecha pago (pendiente extracto MP)</t>
+          <t>Op 175716187231 · CUIL 30536004005 · Banco Comafi · Original 222824.05 · ceil</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">

</xml_diff>